<commit_message>
feat: adding a local files to send to cloud
</commit_message>
<xml_diff>
--- a/components/steam_data_aspen.xlsx
+++ b/components/steam_data_aspen.xlsx
@@ -9,6 +9,9 @@
   <sheets>
     <sheet name="December" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="December1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="December2" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="December3" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="December4" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1389,4 +1392,1432 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Meter 1</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Bypass</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Meter Blue</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Meter Red</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Steam Flow Meter</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Aspen</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>12/03/25</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>12/02/25</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>92</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>12/01/25</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>11/30/25</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>76</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>11/29/25</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>81</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>11/27/25</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>120379</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>30025</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>10025</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>80520100</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>71327</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>11/23/25</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>120371</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>30007</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>10017</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>80517594</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>71316</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>11/23/25</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>120372</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>30010</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>10019</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>80518594</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>71318</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>11/23/25</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>120373</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>30012</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>10019</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>80519594</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>71319</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>11/22/25</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>120003</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>29928</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>9941</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>80268474</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>71145</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>11/19/25</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>119570</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>29845</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>9855</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>79996126</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>70974</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>11/17/25</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>119524</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>29836</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>9836</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>79969750</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>70959</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>08/10/25</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>81</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="C15" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>-66</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>-26</v>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Meter 1</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Bypass</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Meter Blue</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Meter Red</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Steam Flow Meter</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Aspen</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>12/03/25</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>12/02/25</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>92</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>12/01/25</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>11/30/25</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>76</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>11/29/25</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>81</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>11/27/25</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>120379</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>30025</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>10025</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>80520100</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>71327</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>11/23/25</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>120371</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>30007</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>10017</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>80517594</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>71316</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>11/23/25</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>120372</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>30010</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>10019</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>80518594</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>71318</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>11/23/25</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>120373</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>30012</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>10019</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>80519594</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>71319</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>11/22/25</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>120003</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>29928</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>9941</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>80268474</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>71145</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>11/19/25</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>119570</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>29845</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>9855</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>79996126</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>70974</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>11/17/25</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>119524</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>29836</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>9836</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>79969750</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>70959</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>08/10/25</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>81</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="C15" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>-66</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>-26</v>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Meter 1</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Bypass</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Meter Blue</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Meter Red</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Steam Flow Meter</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Aspen</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>12/03/25</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>12/02/25</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>92</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>12/01/25</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>11/30/25</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>76</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>11/29/25</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>81</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>11/27/25</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>120379</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>30025</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>10025</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>80520100</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>71327</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>11/23/25</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>120371</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>30007</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>10017</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>80517594</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>71316</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>11/23/25</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>120372</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>30010</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>10019</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>80518594</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>71318</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>11/23/25</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>120373</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>30012</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>10019</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>80519594</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>71319</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>11/22/25</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>120003</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>29928</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>9941</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>80268474</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>71145</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>11/19/25</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>119570</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>29845</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>9855</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>79996126</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>70974</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>11/17/25</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>119524</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>29836</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>9836</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>79969750</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>70959</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>08/10/25</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>81</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="C15" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>-66</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>-26</v>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>